<commit_message>
Maniac nach Änderungswünschen, alle noch nicht generierten Songs generiert, Blinder-Kaskade
Maniac (Song 30):
- Drum-Intro: Ping-Pong nur auf Bass/Matrix/Gitarre, Lampen mit eigenen kurzen Blindern
- verse 1b: Linien verblassen (progRandomLines mit fadeMillis)
- MANIAC-Text zusätzlich bei Takt 52, 94, 150
- Strobos verschoben (ab 61,5 / bis 73), verse 2b Drop rot
- neue Szene SCENE_CALL_RESPONSE_OFFBEAT (nur auf 2 und 4) für heat und knife 2
- solo a mit mehr Action, Schluss-Blinder auf 160 klingt 2 Takte bis ins Schluss-Schwarz aus
- progPingPong mit Bereich der Bühnenplätze
- songgen.py: Blinder mit carry darf länger sein als sein Part

Außerdem mitgenommen (Stand vom 18.10.2026): Blinder-Kaskade (fxBlinderCascade), Tabellen-Werkzeuge,
neu generierte Songs (Bloody Mary, Don't Stop The Music, Firework, In The Dark, No Roots, Physical,
Such A Shame, Titanium) und neu generierte bestehende Songs, Doku.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/songs/AllTheThingsSheSaid_v1/quelle/struktur.xlsx
+++ b/songs/AllTheThingsSheSaid_v1/quelle/struktur.xlsx
@@ -93,7 +93,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -123,6 +123,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor rgb="FFFFFF00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -136,7 +142,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="42">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -233,6 +239,9 @@
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2726,18 +2735,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G86"/>
+  <dimension ref="A1:H86"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
     <col width="8.5546875" bestFit="1" customWidth="1" style="34" min="1" max="1"/>
     <col width="25.5546875" customWidth="1" style="19" min="2" max="2"/>
     <col width="70" customWidth="1" style="19" min="3" max="3"/>
-    <col width="40" customWidth="1" style="34" min="4" max="4"/>
-    <col width="13.88671875" customWidth="1" min="5" max="5"/>
-    <col width="8.88671875" customWidth="1" min="6" max="6"/>
+    <col width="50" customWidth="1" style="34" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="13.88671875" customWidth="1" min="6" max="6"/>
     <col width="8.88671875" customWidth="1" style="19" min="7" max="7"/>
     <col width="8.88671875" customWidth="1" min="8" max="8"/>
     <col width="8.88671875" customWidth="1" style="19" min="9" max="16384"/>
+    <col width="8.88671875" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2752,6 +2762,7 @@
         </is>
       </c>
       <c r="D1" s="35" t="n"/>
+      <c r="E1" s="35" t="n"/>
     </row>
     <row r="2">
       <c r="B2" s="35" t="inlineStr">
@@ -2763,8 +2774,9 @@
         <v>31</v>
       </c>
       <c r="D2" s="35" t="n"/>
-      <c r="E2" s="39" t="n"/>
+      <c r="E2" s="35" t="n"/>
       <c r="F2" s="39" t="n"/>
+      <c r="G2" s="39" t="n"/>
     </row>
     <row r="3">
       <c r="B3" s="35" t="inlineStr">
@@ -2776,6 +2788,7 @@
         <v>86</v>
       </c>
       <c r="D3" s="35" t="n"/>
+      <c r="E3" s="35" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="36" t="n"/>
@@ -2788,6 +2801,7 @@
         <v>0.375</v>
       </c>
       <c r="D4" s="35" t="n"/>
+      <c r="E4" s="35" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
@@ -2807,15 +2821,20 @@
       </c>
       <c r="D5" s="12" t="inlineStr">
         <is>
+          <t>Alter Effekt (temporär)</t>
+        </is>
+      </c>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
           <t>Änderungswunsch</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="F5" s="11" t="inlineStr">
         <is>
           <t>Energie 0-5</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="G5" s="11" t="inlineStr">
         <is>
           <t>BPM pro Part</t>
         </is>
@@ -2837,14 +2856,15 @@
         </is>
       </c>
       <c r="D6" s="41" t="n"/>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="41" t="n"/>
+      <c r="F6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="5">
+      <c r="G6" s="5">
         <f>$C$3</f>
         <v/>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>ms-Timer startet nicht bei 0, sondern ab StartBit midi-Signal</t>
         </is>
@@ -2867,10 +2887,11 @@
         </is>
       </c>
       <c r="D7" s="41" t="n"/>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="41" t="n"/>
+      <c r="F7" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F7" s="5">
+      <c r="G7" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -2891,10 +2912,11 @@
         </is>
       </c>
       <c r="D8" s="41" t="n"/>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="41" t="n"/>
+      <c r="F8" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F8" s="5">
+      <c r="G8" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -2917,10 +2939,11 @@
         </is>
       </c>
       <c r="D9" s="41" t="n"/>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="41" t="n"/>
+      <c r="F9" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F9" s="5">
+      <c r="G9" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -2942,10 +2965,11 @@
         </is>
       </c>
       <c r="D10" s="41" t="n"/>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="41" t="n"/>
+      <c r="F10" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F10" s="5">
+      <c r="G10" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -2959,18 +2983,25 @@
           <t>verse 1b</t>
         </is>
       </c>
-      <c r="C11" s="41" t="inlineStr">
+      <c r="C11" s="42" t="inlineStr">
+        <is>
+          <t>SCENE_VERSE_PLASMA, Farben SCHEME_ROYAL, Farbwanderung to triad, per 8
+Ausgabe: Übergang fade 1395 ms
+Idee 'etwas gesteigert', energy 2: fließende Farbwolken bringen Bewegung, alles schwillt im Beat leicht an; Blau/Lila wandern nach Pink/Orange und zurück</t>
+        </is>
+      </c>
+      <c r="D11" s="41" t="inlineStr">
         <is>
           <t>SCENE_RAIN, Farben SCHEME_ROYAL, Farbwanderung to triad, per 8
 Ausgabe: Übergang fade 1395 ms
 Idee 'etwas gesteigert', energy 2: fallende Leuchtspuren bringen Bewegung (Regen passt zum Song); Blau/Lila wandern nach Pink/Orange und zurück</t>
         </is>
       </c>
-      <c r="D11" s="41" t="n"/>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="41" t="n"/>
+      <c r="F11" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F11" s="5">
+      <c r="G11" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -2991,10 +3022,11 @@
         </is>
       </c>
       <c r="D12" s="41" t="n"/>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="41" t="n"/>
+      <c r="F12" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F12" s="5">
+      <c r="G12" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3015,10 +3047,11 @@
         </is>
       </c>
       <c r="D13" s="41" t="n"/>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="41" t="n"/>
+      <c r="F13" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F13" s="5">
+      <c r="G13" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3039,10 +3072,11 @@
         </is>
       </c>
       <c r="D14" s="41" t="n"/>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="41" t="n"/>
+      <c r="F14" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="5">
+      <c r="G14" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3065,10 +3099,11 @@
         </is>
       </c>
       <c r="D15" s="41" t="n"/>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="41" t="n"/>
+      <c r="F15" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F15" s="5">
+      <c r="G15" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3090,10 +3125,11 @@
         </is>
       </c>
       <c r="D16" s="41" t="n"/>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="41" t="n"/>
+      <c r="F16" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F16" s="5">
+      <c r="G16" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3114,10 +3150,11 @@
         </is>
       </c>
       <c r="D17" s="41" t="n"/>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="41" t="n"/>
+      <c r="F17" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F17" s="5">
+      <c r="G17" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3140,10 +3177,11 @@
         </is>
       </c>
       <c r="D18" s="41" t="n"/>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="41" t="n"/>
+      <c r="F18" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="5">
+      <c r="G18" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3164,10 +3202,11 @@
         </is>
       </c>
       <c r="D19" s="41" t="n"/>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="41" t="n"/>
+      <c r="F19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F19" s="5">
+      <c r="G19" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3188,10 +3227,11 @@
         </is>
       </c>
       <c r="D20" s="41" t="n"/>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="41" t="n"/>
+      <c r="F20" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F20" s="5">
+      <c r="G20" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3212,10 +3252,11 @@
         </is>
       </c>
       <c r="D21" s="41" t="n"/>
-      <c r="E21" s="5" t="n">
+      <c r="E21" s="41" t="n"/>
+      <c r="F21" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F21" s="5">
+      <c r="G21" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3236,10 +3277,11 @@
         </is>
       </c>
       <c r="D22" s="41" t="n"/>
-      <c r="E22" s="5" t="n">
+      <c r="E22" s="41" t="n"/>
+      <c r="F22" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F22" s="5">
+      <c r="G22" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3262,10 +3304,11 @@
         </is>
       </c>
       <c r="D23" s="41" t="n"/>
-      <c r="E23" s="5" t="n">
+      <c r="E23" s="41" t="n"/>
+      <c r="F23" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F23" s="5">
+      <c r="G23" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3287,10 +3330,11 @@
         </is>
       </c>
       <c r="D24" s="41" t="n"/>
-      <c r="E24" s="5" t="n">
+      <c r="E24" s="41" t="n"/>
+      <c r="F24" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="5">
+      <c r="G24" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3312,10 +3356,11 @@
         </is>
       </c>
       <c r="D25" s="41" t="n"/>
-      <c r="E25" s="5" t="n">
+      <c r="E25" s="41" t="n"/>
+      <c r="F25" s="5" t="n">
         <v>2</v>
       </c>
-      <c r="F25" s="5">
+      <c r="G25" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3336,10 +3381,11 @@
         </is>
       </c>
       <c r="D26" s="41" t="n"/>
-      <c r="E26" s="5" t="n">
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="F26" s="5">
+      <c r="G26" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3360,10 +3406,11 @@
         </is>
       </c>
       <c r="D27" s="41" t="n"/>
-      <c r="E27" s="5" t="n">
+      <c r="E27" s="41" t="n"/>
+      <c r="F27" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F27" s="5">
+      <c r="G27" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3384,10 +3431,11 @@
         </is>
       </c>
       <c r="D28" s="41" t="n"/>
-      <c r="E28" s="5" t="n">
+      <c r="E28" s="41" t="n"/>
+      <c r="F28" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F28" s="5">
+      <c r="G28" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3408,10 +3456,11 @@
         </is>
       </c>
       <c r="D29" s="41" t="n"/>
-      <c r="E29" s="5" t="n">
+      <c r="E29" s="41" t="n"/>
+      <c r="F29" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="F29" s="5">
+      <c r="G29" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3433,10 +3482,11 @@
         </is>
       </c>
       <c r="D30" s="41" t="n"/>
-      <c r="E30" s="5" t="n">
+      <c r="E30" s="41" t="n"/>
+      <c r="F30" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F30" s="5">
+      <c r="G30" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3459,10 +3509,11 @@
         </is>
       </c>
       <c r="D31" s="41" t="n"/>
-      <c r="E31" s="5" t="n">
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F31" s="5">
+      <c r="G31" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3483,10 +3534,11 @@
         </is>
       </c>
       <c r="D32" s="41" t="n"/>
-      <c r="E32" s="5" t="n">
+      <c r="E32" s="41" t="n"/>
+      <c r="F32" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F32" s="5">
+      <c r="G32" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3507,10 +3559,11 @@
         </is>
       </c>
       <c r="D33" s="41" t="n"/>
-      <c r="E33" s="5" t="n">
+      <c r="E33" s="41" t="n"/>
+      <c r="F33" s="5" t="n">
         <v>4</v>
       </c>
-      <c r="F33" s="5">
+      <c r="G33" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3532,10 +3585,11 @@
         </is>
       </c>
       <c r="D34" s="41" t="n"/>
-      <c r="E34" s="5" t="n">
+      <c r="E34" s="41" t="n"/>
+      <c r="F34" s="5" t="n">
         <v>5</v>
       </c>
-      <c r="F34" s="5">
+      <c r="G34" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3557,10 +3611,11 @@
         </is>
       </c>
       <c r="D35" s="41" t="n"/>
-      <c r="E35" s="5" t="n">
+      <c r="E35" s="41" t="n"/>
+      <c r="F35" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="F35" s="5">
+      <c r="G35" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3580,10 +3635,11 @@
         </is>
       </c>
       <c r="D36" s="1" t="n"/>
-      <c r="E36" s="40" t="n">
+      <c r="E36" s="1" t="n"/>
+      <c r="F36" s="40" t="n">
         <v>0</v>
       </c>
-      <c r="F36" s="5">
+      <c r="G36" s="5">
         <f>$C$3</f>
         <v/>
       </c>
@@ -3591,302 +3647,352 @@
     <row r="37">
       <c r="C37" s="1" t="n"/>
       <c r="D37" s="1" t="n"/>
-      <c r="E37" s="40" t="n"/>
+      <c r="E37" s="1" t="n"/>
       <c r="F37" s="40" t="n"/>
+      <c r="G37" s="40" t="n"/>
     </row>
     <row r="38">
       <c r="C38" s="1" t="n"/>
       <c r="D38" s="1" t="n"/>
-      <c r="E38" s="40" t="n"/>
+      <c r="E38" s="1" t="n"/>
       <c r="F38" s="40" t="n"/>
+      <c r="G38" s="40" t="n"/>
     </row>
     <row r="39">
       <c r="C39" s="1" t="n"/>
       <c r="D39" s="1" t="n"/>
-      <c r="E39" s="40" t="n"/>
+      <c r="E39" s="1" t="n"/>
       <c r="F39" s="40" t="n"/>
+      <c r="G39" s="40" t="n"/>
     </row>
     <row r="40">
       <c r="C40" s="1" t="n"/>
       <c r="D40" s="1" t="n"/>
-      <c r="E40" s="40" t="n"/>
+      <c r="E40" s="1" t="n"/>
       <c r="F40" s="40" t="n"/>
+      <c r="G40" s="40" t="n"/>
     </row>
     <row r="41">
       <c r="C41" s="1" t="n"/>
       <c r="D41" s="1" t="n"/>
-      <c r="E41" s="40" t="n"/>
+      <c r="E41" s="1" t="n"/>
       <c r="F41" s="40" t="n"/>
+      <c r="G41" s="40" t="n"/>
     </row>
     <row r="42">
       <c r="C42" s="1" t="n"/>
       <c r="D42" s="1" t="n"/>
-      <c r="E42" s="40" t="n"/>
+      <c r="E42" s="1" t="n"/>
       <c r="F42" s="40" t="n"/>
+      <c r="G42" s="40" t="n"/>
     </row>
     <row r="43">
       <c r="C43" s="1" t="n"/>
       <c r="D43" s="1" t="n"/>
-      <c r="E43" s="40" t="n"/>
+      <c r="E43" s="1" t="n"/>
       <c r="F43" s="40" t="n"/>
+      <c r="G43" s="40" t="n"/>
     </row>
     <row r="44">
       <c r="C44" s="1" t="n"/>
       <c r="D44" s="1" t="n"/>
-      <c r="E44" s="40" t="n"/>
+      <c r="E44" s="1" t="n"/>
       <c r="F44" s="40" t="n"/>
+      <c r="G44" s="40" t="n"/>
     </row>
     <row r="45">
       <c r="C45" s="1" t="n"/>
       <c r="D45" s="1" t="n"/>
-      <c r="E45" s="40" t="n"/>
+      <c r="E45" s="1" t="n"/>
       <c r="F45" s="40" t="n"/>
+      <c r="G45" s="40" t="n"/>
     </row>
     <row r="46">
       <c r="C46" s="1" t="n"/>
       <c r="D46" s="1" t="n"/>
-      <c r="E46" s="40" t="n"/>
+      <c r="E46" s="1" t="n"/>
       <c r="F46" s="40" t="n"/>
+      <c r="G46" s="40" t="n"/>
     </row>
     <row r="47">
       <c r="C47" s="1" t="n"/>
       <c r="D47" s="1" t="n"/>
-      <c r="E47" s="40" t="n"/>
+      <c r="E47" s="1" t="n"/>
       <c r="F47" s="40" t="n"/>
+      <c r="G47" s="40" t="n"/>
     </row>
     <row r="48">
       <c r="C48" s="1" t="n"/>
       <c r="D48" s="1" t="n"/>
-      <c r="E48" s="40" t="n"/>
+      <c r="E48" s="1" t="n"/>
       <c r="F48" s="40" t="n"/>
+      <c r="G48" s="40" t="n"/>
     </row>
     <row r="49">
       <c r="C49" s="1" t="n"/>
       <c r="D49" s="1" t="n"/>
-      <c r="E49" s="40" t="n"/>
+      <c r="E49" s="1" t="n"/>
       <c r="F49" s="40" t="n"/>
+      <c r="G49" s="40" t="n"/>
     </row>
     <row r="50">
       <c r="C50" s="1" t="n"/>
       <c r="D50" s="1" t="n"/>
-      <c r="E50" s="40" t="n"/>
+      <c r="E50" s="1" t="n"/>
       <c r="F50" s="40" t="n"/>
+      <c r="G50" s="40" t="n"/>
     </row>
     <row r="51">
       <c r="C51" s="1" t="n"/>
       <c r="D51" s="1" t="n"/>
-      <c r="E51" s="40" t="n"/>
+      <c r="E51" s="1" t="n"/>
       <c r="F51" s="40" t="n"/>
+      <c r="G51" s="40" t="n"/>
     </row>
     <row r="52">
       <c r="C52" s="1" t="n"/>
       <c r="D52" s="1" t="n"/>
-      <c r="E52" s="40" t="n"/>
+      <c r="E52" s="1" t="n"/>
       <c r="F52" s="40" t="n"/>
+      <c r="G52" s="40" t="n"/>
     </row>
     <row r="53">
       <c r="C53" s="1" t="n"/>
       <c r="D53" s="1" t="n"/>
-      <c r="E53" s="40" t="n"/>
+      <c r="E53" s="1" t="n"/>
       <c r="F53" s="40" t="n"/>
+      <c r="G53" s="40" t="n"/>
     </row>
     <row r="54">
       <c r="C54" s="1" t="n"/>
       <c r="D54" s="1" t="n"/>
-      <c r="E54" s="40" t="n"/>
+      <c r="E54" s="1" t="n"/>
       <c r="F54" s="40" t="n"/>
+      <c r="G54" s="40" t="n"/>
     </row>
     <row r="55">
       <c r="C55" s="1" t="n"/>
       <c r="D55" s="1" t="n"/>
-      <c r="E55" s="40" t="n"/>
+      <c r="E55" s="1" t="n"/>
       <c r="F55" s="40" t="n"/>
+      <c r="G55" s="40" t="n"/>
     </row>
     <row r="56">
       <c r="C56" s="1" t="n"/>
       <c r="D56" s="1" t="n"/>
-      <c r="E56" s="40" t="n"/>
+      <c r="E56" s="1" t="n"/>
       <c r="F56" s="40" t="n"/>
+      <c r="G56" s="40" t="n"/>
     </row>
     <row r="57">
       <c r="C57" s="1" t="n"/>
       <c r="D57" s="1" t="n"/>
-      <c r="E57" s="40" t="n"/>
+      <c r="E57" s="1" t="n"/>
       <c r="F57" s="40" t="n"/>
+      <c r="G57" s="40" t="n"/>
     </row>
     <row r="58">
       <c r="C58" s="1" t="n"/>
       <c r="D58" s="1" t="n"/>
-      <c r="E58" s="40" t="n"/>
+      <c r="E58" s="1" t="n"/>
       <c r="F58" s="40" t="n"/>
+      <c r="G58" s="40" t="n"/>
     </row>
     <row r="59">
       <c r="C59" s="1" t="n"/>
       <c r="D59" s="1" t="n"/>
-      <c r="E59" s="40" t="n"/>
+      <c r="E59" s="1" t="n"/>
       <c r="F59" s="40" t="n"/>
+      <c r="G59" s="40" t="n"/>
     </row>
     <row r="60">
       <c r="C60" s="1" t="n"/>
       <c r="D60" s="1" t="n"/>
-      <c r="E60" s="40" t="n"/>
+      <c r="E60" s="1" t="n"/>
       <c r="F60" s="40" t="n"/>
+      <c r="G60" s="40" t="n"/>
     </row>
     <row r="61">
       <c r="C61" s="1" t="n"/>
       <c r="D61" s="1" t="n"/>
-      <c r="E61" s="40" t="n"/>
+      <c r="E61" s="1" t="n"/>
       <c r="F61" s="40" t="n"/>
+      <c r="G61" s="40" t="n"/>
     </row>
     <row r="62">
       <c r="C62" s="1" t="n"/>
       <c r="D62" s="1" t="n"/>
-      <c r="E62" s="40" t="n"/>
+      <c r="E62" s="1" t="n"/>
       <c r="F62" s="40" t="n"/>
+      <c r="G62" s="40" t="n"/>
     </row>
     <row r="63">
       <c r="C63" s="1" t="n"/>
       <c r="D63" s="1" t="n"/>
-      <c r="E63" s="40" t="n"/>
+      <c r="E63" s="1" t="n"/>
       <c r="F63" s="40" t="n"/>
+      <c r="G63" s="40" t="n"/>
     </row>
     <row r="64">
       <c r="C64" s="1" t="n"/>
       <c r="D64" s="1" t="n"/>
-      <c r="E64" s="40" t="n"/>
+      <c r="E64" s="1" t="n"/>
       <c r="F64" s="40" t="n"/>
+      <c r="G64" s="40" t="n"/>
     </row>
     <row r="65">
       <c r="C65" s="1" t="n"/>
       <c r="D65" s="1" t="n"/>
-      <c r="E65" s="40" t="n"/>
+      <c r="E65" s="1" t="n"/>
       <c r="F65" s="40" t="n"/>
+      <c r="G65" s="40" t="n"/>
     </row>
     <row r="66">
       <c r="C66" s="1" t="n"/>
       <c r="D66" s="1" t="n"/>
-      <c r="E66" s="40" t="n"/>
+      <c r="E66" s="1" t="n"/>
       <c r="F66" s="40" t="n"/>
+      <c r="G66" s="40" t="n"/>
     </row>
     <row r="67">
       <c r="C67" s="1" t="n"/>
       <c r="D67" s="1" t="n"/>
-      <c r="E67" s="40" t="n"/>
+      <c r="E67" s="1" t="n"/>
       <c r="F67" s="40" t="n"/>
+      <c r="G67" s="40" t="n"/>
     </row>
     <row r="68">
       <c r="C68" s="1" t="n"/>
       <c r="D68" s="1" t="n"/>
-      <c r="E68" s="40" t="n"/>
+      <c r="E68" s="1" t="n"/>
       <c r="F68" s="40" t="n"/>
+      <c r="G68" s="40" t="n"/>
     </row>
     <row r="69">
       <c r="C69" s="1" t="n"/>
       <c r="D69" s="1" t="n"/>
-      <c r="E69" s="40" t="n"/>
+      <c r="E69" s="1" t="n"/>
       <c r="F69" s="40" t="n"/>
+      <c r="G69" s="40" t="n"/>
     </row>
     <row r="70">
       <c r="C70" s="1" t="n"/>
       <c r="D70" s="1" t="n"/>
-      <c r="E70" s="40" t="n"/>
+      <c r="E70" s="1" t="n"/>
       <c r="F70" s="40" t="n"/>
+      <c r="G70" s="40" t="n"/>
     </row>
     <row r="71">
       <c r="C71" s="1" t="n"/>
       <c r="D71" s="1" t="n"/>
-      <c r="E71" s="40" t="n"/>
+      <c r="E71" s="1" t="n"/>
       <c r="F71" s="40" t="n"/>
+      <c r="G71" s="40" t="n"/>
     </row>
     <row r="72">
       <c r="C72" s="1" t="n"/>
       <c r="D72" s="1" t="n"/>
-      <c r="E72" s="40" t="n"/>
+      <c r="E72" s="1" t="n"/>
       <c r="F72" s="40" t="n"/>
+      <c r="G72" s="40" t="n"/>
     </row>
     <row r="73">
       <c r="C73" s="1" t="n"/>
       <c r="D73" s="1" t="n"/>
-      <c r="E73" s="40" t="n"/>
+      <c r="E73" s="1" t="n"/>
       <c r="F73" s="40" t="n"/>
+      <c r="G73" s="40" t="n"/>
     </row>
     <row r="74">
       <c r="C74" s="1" t="n"/>
       <c r="D74" s="1" t="n"/>
-      <c r="E74" s="40" t="n"/>
+      <c r="E74" s="1" t="n"/>
       <c r="F74" s="40" t="n"/>
+      <c r="G74" s="40" t="n"/>
     </row>
     <row r="75">
       <c r="C75" s="1" t="n"/>
       <c r="D75" s="1" t="n"/>
-      <c r="E75" s="40" t="n"/>
+      <c r="E75" s="1" t="n"/>
       <c r="F75" s="40" t="n"/>
+      <c r="G75" s="40" t="n"/>
     </row>
     <row r="76">
       <c r="C76" s="1" t="n"/>
       <c r="D76" s="1" t="n"/>
-      <c r="E76" s="40" t="n"/>
+      <c r="E76" s="1" t="n"/>
       <c r="F76" s="40" t="n"/>
+      <c r="G76" s="40" t="n"/>
     </row>
     <row r="77">
       <c r="C77" s="1" t="n"/>
       <c r="D77" s="1" t="n"/>
-      <c r="E77" s="40" t="n"/>
+      <c r="E77" s="1" t="n"/>
       <c r="F77" s="40" t="n"/>
+      <c r="G77" s="40" t="n"/>
     </row>
     <row r="78">
       <c r="C78" s="1" t="n"/>
       <c r="D78" s="1" t="n"/>
-      <c r="E78" s="40" t="n"/>
+      <c r="E78" s="1" t="n"/>
       <c r="F78" s="40" t="n"/>
+      <c r="G78" s="40" t="n"/>
     </row>
     <row r="79">
       <c r="C79" s="1" t="n"/>
       <c r="D79" s="1" t="n"/>
-      <c r="E79" s="40" t="n"/>
+      <c r="E79" s="1" t="n"/>
       <c r="F79" s="40" t="n"/>
+      <c r="G79" s="40" t="n"/>
     </row>
     <row r="80">
       <c r="C80" s="1" t="n"/>
       <c r="D80" s="1" t="n"/>
-      <c r="E80" s="40" t="n"/>
+      <c r="E80" s="1" t="n"/>
       <c r="F80" s="40" t="n"/>
+      <c r="G80" s="40" t="n"/>
     </row>
     <row r="81">
       <c r="C81" s="1" t="n"/>
       <c r="D81" s="1" t="n"/>
-      <c r="E81" s="40" t="n"/>
+      <c r="E81" s="1" t="n"/>
       <c r="F81" s="40" t="n"/>
+      <c r="G81" s="40" t="n"/>
     </row>
     <row r="82">
       <c r="C82" s="1" t="n"/>
       <c r="D82" s="1" t="n"/>
-      <c r="E82" s="40" t="n"/>
+      <c r="E82" s="1" t="n"/>
       <c r="F82" s="40" t="n"/>
+      <c r="G82" s="40" t="n"/>
     </row>
     <row r="83">
       <c r="C83" s="1" t="n"/>
       <c r="D83" s="1" t="n"/>
-      <c r="E83" s="40" t="n"/>
+      <c r="E83" s="1" t="n"/>
       <c r="F83" s="40" t="n"/>
+      <c r="G83" s="40" t="n"/>
     </row>
     <row r="84">
       <c r="C84" s="1" t="n"/>
       <c r="D84" s="1" t="n"/>
-      <c r="E84" s="40" t="n"/>
+      <c r="E84" s="1" t="n"/>
       <c r="F84" s="40" t="n"/>
+      <c r="G84" s="40" t="n"/>
     </row>
     <row r="85">
       <c r="C85" s="1" t="n"/>
       <c r="D85" s="1" t="n"/>
-      <c r="E85" s="40" t="n"/>
+      <c r="E85" s="1" t="n"/>
       <c r="F85" s="40" t="n"/>
+      <c r="G85" s="40" t="n"/>
     </row>
     <row r="86">
       <c r="C86" s="1" t="n"/>
       <c r="D86" s="1" t="n"/>
-      <c r="E86" s="40" t="n"/>
+      <c r="E86" s="1" t="n"/>
       <c r="F86" s="40" t="n"/>
+      <c r="G86" s="40" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>